<commit_message>
fix(resume-screen): address munmiu review on example tests
Stop asserting browser CLIs are absent so machines with ego-browser
or agent-browser still pass. Resolve File hyperlinks relative to the
workbook (resumes/<name>.md). Write unittest xlsx under tempfile;
regenerate the committed workbook only via build-example-workbook.py.
Replace the tautological Total assert with a real factor-sum check.

Co-authored-by: Duc Nguyen <me@vanducng.dev>
</commit_message>
<xml_diff>
--- a/skills/resume-screen/examples/sample-scorecard.xlsx
+++ b/skills/resume-screen/examples/sample-scorecard.xlsx
@@ -219,7 +219,7 @@
         </is>
       </c>
       <c r="C2">
-        <f>HYPERLINK("examples/resumes/jordan-hale.md","jordan-hale.md")</f>
+        <f>HYPERLINK("resumes/jordan-hale.md","jordan-hale.md")</f>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -357,7 +357,7 @@
         </is>
       </c>
       <c r="C3">
-        <f>HYPERLINK("examples/resumes/morgan-ellis.md","morgan-ellis.md")</f>
+        <f>HYPERLINK("resumes/morgan-ellis.md","morgan-ellis.md")</f>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="C4">
-        <f>HYPERLINK("examples/resumes/avery-kim.md","avery-kim.md")</f>
+        <f>HYPERLINK("resumes/avery-kim.md","avery-kim.md")</f>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="C5">
-        <f>HYPERLINK("examples/resumes/riley-chen.md","riley-chen.md")</f>
+        <f>HYPERLINK("resumes/riley-chen.md","riley-chen.md")</f>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">examples/sample-jd.md</t>
+          <t xml:space="preserve">sample-jd.md</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-14T10:18:56Z</t>
+          <t xml:space="preserve">2026-08-14T10:36:52Z</t>
         </is>
       </c>
     </row>

</xml_diff>